<commit_message>
Add a Note column, and stop a re-run from wiping a filled-in sheet
Note is the last column, free text, never parsed — contributors can leave
remarks for each other without it affecting the newsletter. The importer finds
its columns by header name, so the extra column changes nothing for it.

Re-running the migration on a sheet already in master format would have
destroyed it: read_old() looks for a field key in column A, which holds Sr No.
there, so nothing matched and every Content cell came back empty. It now
recognises the master layout, keeps the Content and Notes already filled in,
and says so instead of silently emptying a month's work.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/master_template.xlsx
+++ b/master_template.xlsx
@@ -597,7 +597,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -606,6 +606,7 @@
     <col width="62" customWidth="1" min="4" max="4"/>
     <col width="26" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -681,6 +682,11 @@
           <t>Field</t>
         </is>
       </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="4" t="inlineStr"/>
@@ -697,6 +703,7 @@
           <t>month</t>
         </is>
       </c>
+      <c r="G9" s="5" t="n"/>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="4" t="inlineStr"/>
@@ -713,6 +720,7 @@
           <t>year</t>
         </is>
       </c>
+      <c r="G10" s="5" t="n"/>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="4" t="n">
@@ -739,6 +747,7 @@
           <t>ceo_message</t>
         </is>
       </c>
+      <c r="G11" s="5" t="n"/>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="4" t="inlineStr"/>
@@ -759,6 +768,7 @@
           <t>ceo_name</t>
         </is>
       </c>
+      <c r="G12" s="5" t="n"/>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="4" t="inlineStr"/>
@@ -779,6 +789,7 @@
           <t>ceo_title</t>
         </is>
       </c>
+      <c r="G13" s="5" t="n"/>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="4" t="n">
@@ -805,6 +816,7 @@
           <t>campaign_banner</t>
         </is>
       </c>
+      <c r="G14" s="5" t="n"/>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="4" t="n">
@@ -831,6 +843,7 @@
           <t>expo</t>
         </is>
       </c>
+      <c r="G15" s="5" t="n"/>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="4" t="n">
@@ -857,6 +870,7 @@
           <t>new_customer</t>
         </is>
       </c>
+      <c r="G16" s="5" t="n"/>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="4" t="n">
@@ -883,6 +897,7 @@
           <t>delivery</t>
         </is>
       </c>
+      <c r="G17" s="5" t="n"/>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="4" t="n">
@@ -909,6 +924,7 @@
           <t>excellence</t>
         </is>
       </c>
+      <c r="G18" s="5" t="n"/>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="4" t="n">
@@ -935,6 +951,7 @@
           <t>excellence</t>
         </is>
       </c>
+      <c r="G19" s="5" t="n"/>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="4" t="n">
@@ -961,6 +978,7 @@
           <t>hr_event1</t>
         </is>
       </c>
+      <c r="G20" s="5" t="n"/>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="4" t="n">
@@ -987,6 +1005,7 @@
           <t>hr_event2</t>
         </is>
       </c>
+      <c r="G21" s="5" t="n"/>
     </row>
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="4" t="n">
@@ -1013,6 +1032,7 @@
           <t>hr_event3</t>
         </is>
       </c>
+      <c r="G22" s="5" t="n"/>
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="4" t="n">
@@ -1039,6 +1059,7 @@
           <t>hr_wellness_banner</t>
         </is>
       </c>
+      <c r="G23" s="5" t="n"/>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="4" t="n">
@@ -1065,6 +1086,7 @@
           <t>award</t>
         </is>
       </c>
+      <c r="G24" s="5" t="n"/>
     </row>
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="4" t="n">
@@ -1091,6 +1113,7 @@
           <t>new_joinee</t>
         </is>
       </c>
+      <c r="G25" s="5" t="n"/>
     </row>
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="4" t="n">
@@ -1113,6 +1136,7 @@
           <t>anniversary</t>
         </is>
       </c>
+      <c r="G26" s="5" t="n"/>
     </row>
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="4" t="n">
@@ -1139,6 +1163,7 @@
           <t>employee_certification</t>
         </is>
       </c>
+      <c r="G27" s="5" t="n"/>
     </row>
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="4" t="n">
@@ -1161,6 +1186,7 @@
           <t>new_openings_sheet</t>
         </is>
       </c>
+      <c r="G28" s="5" t="n"/>
     </row>
     <row r="29" ht="30" customHeight="1">
       <c r="A29" s="4" t="n">
@@ -1187,6 +1213,7 @@
           <t>employee_training</t>
         </is>
       </c>
+      <c r="G29" s="5" t="n"/>
     </row>
     <row r="30" ht="30" customHeight="1">
       <c r="A30" s="4" t="n">
@@ -1213,6 +1240,7 @@
           <t>employee_workshop</t>
         </is>
       </c>
+      <c r="G30" s="5" t="n"/>
     </row>
     <row r="31" ht="30" customHeight="1">
       <c r="A31" s="4" t="n">
@@ -1239,6 +1267,7 @@
           <t>new_announcement</t>
         </is>
       </c>
+      <c r="G31" s="5" t="n"/>
     </row>
     <row r="32" ht="30" customHeight="1">
       <c r="A32" s="4" t="n">
@@ -1265,15 +1294,16 @@
           <t>marketing_highlights</t>
         </is>
       </c>
+      <c r="G32" s="5" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A5:F5"/>
-    <mergeCell ref="A6:F6"/>
-    <mergeCell ref="A4:F4"/>
-    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="A6:G6"/>
+    <mergeCell ref="A4:G4"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A5:G5"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation sqref="D9:D32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Content" prompt="Type the content, leave blank, or write NA to drop this section." type="list">

</xml_diff>

<commit_message>
Put the essential guidance in plain cells so it survives a copy-paste
Per-row hints lived only in cell comments, which are dropped when the sheet is
copy-pasted into Google Sheets — along with the fills, borders and column
widths. The instructions block at the top is plain cells and does survive, so
it now carries everything that actually matters: the NA rule, the photo folder
and filename conventions, the HEIC warning, and the Tab-separated shapes for
the Work Anniversary, New Openings and Marketing paste-in lists. The comments
stay as a convenience where they do survive.

Confirmed the importer only ever reads cell values: a copy with every fill,
font, border, width, merge, comment and validation stripped parses identically
- same month, same 9 anniversary groups, same 3 openings, same sections. Lost
formatting is cosmetic, never a broken run.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/master_template.xlsx
+++ b/master_template.xlsx
@@ -184,122 +184,122 @@
     <author>Newsletter</author>
   </authors>
   <commentList>
-    <comment ref="D9" authorId="0" shapeId="0">
+    <comment ref="D12" authorId="0" shapeId="0">
       <text>
         <t>e.g. July</t>
       </text>
     </comment>
-    <comment ref="D10" authorId="0" shapeId="0">
+    <comment ref="D13" authorId="0" shapeId="0">
       <text>
         <t>e.g. 2026</t>
       </text>
     </comment>
-    <comment ref="D11" authorId="0" shapeId="0">
+    <comment ref="D14" authorId="0" shapeId="0">
       <text>
         <t>The CXO's message. Their photo goes in the folder.</t>
       </text>
     </comment>
-    <comment ref="D12" authorId="0" shapeId="0">
+    <comment ref="D15" authorId="0" shapeId="0">
       <text>
         <t>Rarely changes, e.g. Maulik Shah</t>
       </text>
     </comment>
-    <comment ref="D13" authorId="0" shapeId="0">
+    <comment ref="D16" authorId="0" shapeId="0">
       <text>
         <t>Rarely changes, e.g. Founder &amp; CEO</t>
       </text>
     </comment>
-    <comment ref="D14" authorId="0" shapeId="0">
+    <comment ref="D17" authorId="0" shapeId="0">
       <text>
         <t>Banner image goes in the folder. Leave blank, or NA to drop.</t>
       </text>
     </comment>
-    <comment ref="D15" authorId="0" shapeId="0">
+    <comment ref="D18" authorId="0" shapeId="0">
       <text>
         <t>Optional heading. Photos go in the folder.</t>
       </text>
     </comment>
-    <comment ref="D16" authorId="0" shapeId="0">
+    <comment ref="D19" authorId="0" shapeId="0">
       <text>
         <t>Logos go in the folder, any filenames.</t>
       </text>
     </comment>
-    <comment ref="D17" authorId="0" shapeId="0">
+    <comment ref="D20" authorId="0" shapeId="0">
       <text>
         <t>The write-up. Client logo goes in the folder.</t>
       </text>
     </comment>
-    <comment ref="D18" authorId="0" shapeId="0">
+    <comment ref="D21" authorId="0" shapeId="0">
       <text>
         <t>The quote. Client logo goes in the folder.</t>
       </text>
     </comment>
-    <comment ref="D19" authorId="0" shapeId="0">
+    <comment ref="D22" authorId="0" shapeId="0">
       <text>
         <t>A second quote, same as above.</t>
       </text>
     </comment>
-    <comment ref="D20" authorId="0" shapeId="0">
+    <comment ref="D23" authorId="0" shapeId="0">
       <text>
         <t>Event name. Photos go in the folder.</t>
       </text>
     </comment>
-    <comment ref="D21" authorId="0" shapeId="0">
+    <comment ref="D24" authorId="0" shapeId="0">
       <text>
         <t>Second event, if there is one.</t>
       </text>
     </comment>
-    <comment ref="D22" authorId="0" shapeId="0">
+    <comment ref="D25" authorId="0" shapeId="0">
       <text>
         <t>Third event, if there is one.</t>
       </text>
     </comment>
-    <comment ref="D23" authorId="0" shapeId="0">
+    <comment ref="D26" authorId="0" shapeId="0">
       <text>
         <t>Heading. Banner image goes in the folder.</t>
       </text>
     </comment>
-    <comment ref="D24" authorId="0" shapeId="0">
+    <comment ref="D27" authorId="0" shapeId="0">
       <text>
         <t>Names come from the filenames -- see the note below.</t>
       </text>
     </comment>
-    <comment ref="D25" authorId="0" shapeId="0">
+    <comment ref="D28" authorId="0" shapeId="0">
       <text>
         <t>Names come from the filenames -- see the note below.</t>
       </text>
     </comment>
-    <comment ref="D26" authorId="0" shapeId="0">
+    <comment ref="D29" authorId="0" shapeId="0">
       <text>
         <t>Paste from your sheet: Name &lt;tab&gt; 5 years, one per line.</t>
       </text>
     </comment>
-    <comment ref="D27" authorId="0" shapeId="0">
+    <comment ref="D30" authorId="0" shapeId="0">
       <text>
         <t>Certificate images go in the folder.</t>
       </text>
     </comment>
-    <comment ref="D28" authorId="0" shapeId="0">
+    <comment ref="D31" authorId="0" shapeId="0">
       <text>
         <t>Paste with header: Position &lt;tab&gt; Experience &lt;tab&gt; Opening.</t>
       </text>
     </comment>
-    <comment ref="D29" authorId="0" shapeId="0">
+    <comment ref="D32" authorId="0" shapeId="0">
       <text>
         <t>Optional heading. Photos go in the folder.</t>
       </text>
     </comment>
-    <comment ref="D30" authorId="0" shapeId="0">
+    <comment ref="D33" authorId="0" shapeId="0">
       <text>
         <t>Optional heading. Photos go in the folder.</t>
       </text>
     </comment>
-    <comment ref="D31" authorId="0" shapeId="0">
+    <comment ref="D34" authorId="0" shapeId="0">
       <text>
         <t>Event name. Banner goes in the folder.</t>
       </text>
     </comment>
-    <comment ref="D32" authorId="0" shapeId="0">
+    <comment ref="D35" authorId="0" shapeId="0">
       <text>
         <t>One per line: Title &lt;tab&gt; https://link</t>
       </text>
@@ -597,7 +597,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -612,160 +612,116 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>BIZTECH NEWSLETTER — fill in the Content column only.</t>
+          <t>BIZTECH NEWSLETTER — fill in the Content column only. Leave the grey Photos Folder / Field columns alone.</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Leave Content blank, or write NA, if a section has nothing this month — it is then left out of the newsletter entirely.</t>
+          <t>Nothing this month? Leave Content blank or write NA — that section is then left out of the newsletter entirely.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Photos: drop them into the folder named in 'Photos Folder'. No links needed.</t>
+          <t>PHOTOS: drop them straight into the folder named in 'Photos Folder'. No links needed. Order follows the filename, so prefix 01, 02, … where it matters.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>R &amp; R filenames:      01 - Award Title - Person Name - Designation.jpg   (repeat the title to group people under one award)</t>
+          <t xml:space="preserve">        R &amp; R filename:       01 - Award Title - Person Name - Designation.jpg   (repeat the award title to group several people under one award)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>New Joiners filenames: Person Name - Designation.jpg</t>
+          <t xml:space="preserve">        New Joiners filename: Person Name - Designation.jpg          iPhone HEIC photos must be re-saved as PNG or JPEG first — renaming them is not enough.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Order inside a folder follows the filename, so prefix 01, 02, … where it matters. iPhone HEIC photos must be saved as PNG/JPEG first.</t>
+          <t>PASTE-IN LISTS (one per line, Tab between the parts — paste straight from another sheet):</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        Work Anniversary:  Person Name &lt;Tab&gt; 5 years</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        New Openings:      Position &lt;Tab&gt; Experience &lt;Tab&gt; Opening        (keep the header line)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        Marketing:         Blog Title &lt;Tab&gt; https://link</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>Sr No.</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>Newsletter Sections</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>POC</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D11" s="3" t="inlineStr">
         <is>
           <t>Content</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E11" s="3" t="inlineStr">
         <is>
           <t>Photos Folder</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="F11" s="3" t="inlineStr">
         <is>
           <t>Field</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="G11" s="3" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
-    </row>
-    <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="4" t="inlineStr"/>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>Newsletter Month</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr"/>
-      <c r="D9" s="5" t="n"/>
-      <c r="E9" s="6" t="inlineStr"/>
-      <c r="F9" s="6" t="inlineStr">
-        <is>
-          <t>month</t>
-        </is>
-      </c>
-      <c r="G9" s="5" t="n"/>
-    </row>
-    <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="4" t="inlineStr"/>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>Newsletter Year</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr"/>
-      <c r="D10" s="5" t="n"/>
-      <c r="E10" s="6" t="inlineStr"/>
-      <c r="F10" s="6" t="inlineStr">
-        <is>
-          <t>year</t>
-        </is>
-      </c>
-      <c r="G10" s="5" t="n"/>
-    </row>
-    <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>Message from CXO's Desk</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>Vedanshi</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="n"/>
-      <c r="E11" s="6" t="inlineStr">
-        <is>
-          <t>Row Data/ceo</t>
-        </is>
-      </c>
-      <c r="F11" s="6" t="inlineStr">
-        <is>
-          <t>ceo_message</t>
-        </is>
-      </c>
-      <c r="G11" s="5" t="n"/>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="4" t="inlineStr"/>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   ↳ CXO Name</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>Vedanshi</t>
-        </is>
-      </c>
+          <t>Newsletter Month</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr"/>
       <c r="D12" s="5" t="n"/>
       <c r="E12" s="6" t="inlineStr"/>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>ceo_name</t>
+          <t>month</t>
         </is>
       </c>
       <c r="G12" s="5" t="n"/>
@@ -774,300 +730,284 @@
       <c r="A13" s="4" t="inlineStr"/>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   ↳ CXO Title</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>Vedanshi</t>
-        </is>
-      </c>
+          <t>Newsletter Year</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr"/>
       <c r="D13" s="5" t="n"/>
       <c r="E13" s="6" t="inlineStr"/>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t>ceo_title</t>
+          <t>year</t>
         </is>
       </c>
       <c r="G13" s="5" t="n"/>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>ISMS Incident Awareness Banner</t>
+          <t>Message from CXO's Desk</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Pratik</t>
+          <t>Vedanshi</t>
         </is>
       </c>
       <c r="D14" s="5" t="n"/>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>Row Data/campaign_banner</t>
+          <t>Row Data/ceo</t>
         </is>
       </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
-          <t>campaign_banner</t>
+          <t>ceo_message</t>
         </is>
       </c>
       <c r="G14" s="5" t="n"/>
     </row>
     <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="4" t="n">
-        <v>3</v>
-      </c>
+      <c r="A15" s="4" t="inlineStr"/>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Monthly Company Expo/Exhibition Photos</t>
+          <t xml:space="preserve">   ↳ CXO Name</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Parth Pandya</t>
+          <t>Vedanshi</t>
         </is>
       </c>
       <c r="D15" s="5" t="n"/>
-      <c r="E15" s="6" t="inlineStr">
-        <is>
-          <t>Row Data/expo</t>
-        </is>
-      </c>
+      <c r="E15" s="6" t="inlineStr"/>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>expo</t>
+          <t>ceo_name</t>
         </is>
       </c>
       <c r="G15" s="5" t="n"/>
     </row>
     <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="4" t="n">
-        <v>4</v>
-      </c>
+      <c r="A16" s="4" t="inlineStr"/>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>New Logos Added (New Clients/Projects)</t>
+          <t xml:space="preserve">   ↳ CXO Title</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Pratik</t>
+          <t>Vedanshi</t>
         </is>
       </c>
       <c r="D16" s="5" t="n"/>
-      <c r="E16" s="6" t="inlineStr">
-        <is>
-          <t>Row Data/new_customer</t>
-        </is>
-      </c>
+      <c r="E16" s="6" t="inlineStr"/>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t>new_customer</t>
+          <t>ceo_title</t>
         </is>
       </c>
       <c r="G16" s="5" t="n"/>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Delivery Insights (If any)</t>
+          <t>ISMS Incident Awareness Banner</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Manish &amp; Jay</t>
+          <t>Pratik</t>
         </is>
       </c>
       <c r="D17" s="5" t="n"/>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>Row Data/delivery</t>
+          <t>Row Data/campaign_banner</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
-          <t>delivery</t>
+          <t>campaign_banner</t>
         </is>
       </c>
       <c r="G17" s="5" t="n"/>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Response from Client to Employees (If Any)</t>
+          <t>Monthly Company Expo/Exhibition Photos</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Manish &amp; Jay</t>
+          <t>Parth Pandya</t>
         </is>
       </c>
       <c r="D18" s="5" t="n"/>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>Row Data/excellence</t>
+          <t>Row Data/expo</t>
         </is>
       </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>excellence</t>
+          <t>expo</t>
         </is>
       </c>
       <c r="G18" s="5" t="n"/>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="4" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Customer Testimonials (If received)</t>
+          <t>New Logos Added (New Clients/Projects)</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Manish &amp; Jay</t>
+          <t>Pratik</t>
         </is>
       </c>
       <c r="D19" s="5" t="n"/>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>Row Data/excellence</t>
+          <t>Row Data/new_customer</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr">
         <is>
-          <t>excellence</t>
+          <t>new_customer</t>
         </is>
       </c>
       <c r="G19" s="5" t="n"/>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="4" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Monthly HR Events</t>
+          <t>Delivery Insights (If any)</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Nikita</t>
+          <t>Manish &amp; Jay</t>
         </is>
       </c>
       <c r="D20" s="5" t="n"/>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>Row Data/events/event1</t>
+          <t>Row Data/delivery</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr">
         <is>
-          <t>hr_event1</t>
+          <t>delivery</t>
         </is>
       </c>
       <c r="G20" s="5" t="n"/>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="4" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Monthly HR Events (2nd event)</t>
+          <t>Response from Client to Employees (If Any)</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Nikita</t>
+          <t>Manish &amp; Jay</t>
         </is>
       </c>
       <c r="D21" s="5" t="n"/>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>Row Data/events/event2</t>
+          <t>Row Data/excellence</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr">
         <is>
-          <t>hr_event2</t>
+          <t>excellence</t>
         </is>
       </c>
       <c r="G21" s="5" t="n"/>
     </row>
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="4" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Monthly HR Events (3rd event)</t>
+          <t>Customer Testimonials (If received)</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Nikita</t>
+          <t>Manish &amp; Jay</t>
         </is>
       </c>
       <c r="D22" s="5" t="n"/>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>Row Data/events/event3</t>
+          <t>Row Data/excellence</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr">
         <is>
-          <t>hr_event3</t>
+          <t>excellence</t>
         </is>
       </c>
       <c r="G22" s="5" t="n"/>
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="4" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>Wellness &amp; HR Corner</t>
+          <t>Monthly HR Events</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Nikita</t>
         </is>
       </c>
       <c r="D23" s="5" t="n"/>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>Row Data/hr_wellness</t>
+          <t>Row Data/events/event1</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr">
         <is>
-          <t>hr_wellness_banner</t>
+          <t>hr_event1</t>
         </is>
       </c>
       <c r="G23" s="5" t="n"/>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="4" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>R &amp; R</t>
+          <t>Monthly HR Events (2nd event)</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
@@ -1078,23 +1018,23 @@
       <c r="D24" s="5" t="n"/>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t>Row Data/awards</t>
+          <t>Row Data/events/event2</t>
         </is>
       </c>
       <c r="F24" s="6" t="inlineStr">
         <is>
-          <t>award</t>
+          <t>hr_event2</t>
         </is>
       </c>
       <c r="G24" s="5" t="n"/>
     </row>
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="4" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>New Joiners (This Month)</t>
+          <t>Monthly HR Events (3rd event)</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
@@ -1105,46 +1045,50 @@
       <c r="D25" s="5" t="n"/>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>Row Data/new_joinee</t>
+          <t>Row Data/events/event3</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr">
         <is>
-          <t>new_joinee</t>
+          <t>hr_event3</t>
         </is>
       </c>
       <c r="G25" s="5" t="n"/>
     </row>
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="4" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Work Anniversary (This Month)</t>
+          <t>Wellness &amp; HR Corner</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Nikita</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D26" s="5" t="n"/>
-      <c r="E26" s="6" t="inlineStr"/>
+      <c r="E26" s="6" t="inlineStr">
+        <is>
+          <t>Row Data/hr_wellness</t>
+        </is>
+      </c>
       <c r="F26" s="6" t="inlineStr">
         <is>
-          <t>anniversary</t>
+          <t>hr_wellness_banner</t>
         </is>
       </c>
       <c r="G26" s="5" t="n"/>
     </row>
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="4" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>Employee Certifications (This Month)</t>
+          <t>R &amp; R</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
@@ -1155,23 +1099,23 @@
       <c r="D27" s="5" t="n"/>
       <c r="E27" s="6" t="inlineStr">
         <is>
-          <t>Row Data/certification</t>
+          <t>Row Data/awards</t>
         </is>
       </c>
       <c r="F27" s="6" t="inlineStr">
         <is>
-          <t>employee_certification</t>
+          <t>award</t>
         </is>
       </c>
       <c r="G27" s="5" t="n"/>
     </row>
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="4" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>New Openings (This Month)</t>
+          <t>New Joiners (This Month)</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
@@ -1180,21 +1124,25 @@
         </is>
       </c>
       <c r="D28" s="5" t="n"/>
-      <c r="E28" s="6" t="inlineStr"/>
+      <c r="E28" s="6" t="inlineStr">
+        <is>
+          <t>Row Data/new_joinee</t>
+        </is>
+      </c>
       <c r="F28" s="6" t="inlineStr">
         <is>
-          <t>new_openings_sheet</t>
+          <t>new_joinee</t>
         </is>
       </c>
       <c r="G28" s="5" t="n"/>
     </row>
     <row r="29" ht="30" customHeight="1">
       <c r="A29" s="4" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>Employee Training (This Month)</t>
+          <t>Work Anniversary (This Month)</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
@@ -1203,25 +1151,21 @@
         </is>
       </c>
       <c r="D29" s="5" t="n"/>
-      <c r="E29" s="6" t="inlineStr">
-        <is>
-          <t>Row Data/training</t>
-        </is>
-      </c>
+      <c r="E29" s="6" t="inlineStr"/>
       <c r="F29" s="6" t="inlineStr">
         <is>
-          <t>employee_training</t>
+          <t>anniversary</t>
         </is>
       </c>
       <c r="G29" s="5" t="n"/>
     </row>
     <row r="30" ht="30" customHeight="1">
       <c r="A30" s="4" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>Employee Workshop (This Month)</t>
+          <t>Employee Certifications (This Month)</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
@@ -1232,23 +1176,23 @@
       <c r="D30" s="5" t="n"/>
       <c r="E30" s="6" t="inlineStr">
         <is>
-          <t>Row Data/workshop</t>
+          <t>Row Data/certification</t>
         </is>
       </c>
       <c r="F30" s="6" t="inlineStr">
         <is>
-          <t>employee_workshop</t>
+          <t>employee_certification</t>
         </is>
       </c>
       <c r="G30" s="5" t="n"/>
     </row>
     <row r="31" ht="30" customHeight="1">
       <c r="A31" s="4" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>Announcement of any Events</t>
+          <t>New Openings (This Month)</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
@@ -1257,56 +1201,136 @@
         </is>
       </c>
       <c r="D31" s="5" t="n"/>
-      <c r="E31" s="6" t="inlineStr">
-        <is>
-          <t>Row Data/announcement</t>
-        </is>
-      </c>
+      <c r="E31" s="6" t="inlineStr"/>
       <c r="F31" s="6" t="inlineStr">
         <is>
-          <t>new_announcement</t>
+          <t>new_openings_sheet</t>
         </is>
       </c>
       <c r="G31" s="5" t="n"/>
     </row>
     <row r="32" ht="30" customHeight="1">
       <c r="A32" s="4" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>Marketing Highlights (Blogs, Case Studies…)</t>
+          <t>Employee Training (This Month)</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Dhaval</t>
+          <t>Nikita</t>
         </is>
       </c>
       <c r="D32" s="5" t="n"/>
       <c r="E32" s="6" t="inlineStr">
         <is>
+          <t>Row Data/training</t>
+        </is>
+      </c>
+      <c r="F32" s="6" t="inlineStr">
+        <is>
+          <t>employee_training</t>
+        </is>
+      </c>
+      <c r="G32" s="5" t="n"/>
+    </row>
+    <row r="33" ht="30" customHeight="1">
+      <c r="A33" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>Employee Workshop (This Month)</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>Nikita</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="n"/>
+      <c r="E33" s="6" t="inlineStr">
+        <is>
+          <t>Row Data/workshop</t>
+        </is>
+      </c>
+      <c r="F33" s="6" t="inlineStr">
+        <is>
+          <t>employee_workshop</t>
+        </is>
+      </c>
+      <c r="G33" s="5" t="n"/>
+    </row>
+    <row r="34" ht="30" customHeight="1">
+      <c r="A34" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>Announcement of any Events</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>Nikita</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="n"/>
+      <c r="E34" s="6" t="inlineStr">
+        <is>
+          <t>Row Data/announcement</t>
+        </is>
+      </c>
+      <c r="F34" s="6" t="inlineStr">
+        <is>
+          <t>new_announcement</t>
+        </is>
+      </c>
+      <c r="G34" s="5" t="n"/>
+    </row>
+    <row r="35" ht="30" customHeight="1">
+      <c r="A35" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>Marketing Highlights (Blogs, Case Studies…)</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>Dhaval</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="n"/>
+      <c r="E35" s="6" t="inlineStr">
+        <is>
           <t>Row Data/marketing/blogs</t>
         </is>
       </c>
-      <c r="F32" s="6" t="inlineStr">
+      <c r="F35" s="6" t="inlineStr">
         <is>
           <t>marketing_highlights</t>
         </is>
       </c>
-      <c r="G32" s="5" t="n"/>
+      <c r="G35" s="5" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="9">
     <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A9:G9"/>
+    <mergeCell ref="A8:G8"/>
     <mergeCell ref="A3:G3"/>
     <mergeCell ref="A6:G6"/>
     <mergeCell ref="A4:G4"/>
     <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A7:G7"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="D9:D32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Content" prompt="Type the content, leave blank, or write NA to drop this section." type="list">
+    <dataValidation sqref="D12:D35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Content" prompt="Type the content, leave blank, or write NA to drop this section." type="list">
       <formula1>"NA"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>